<commit_message>
fix: added version number to manual and adjusted point annotation order in visualizations.
</commit_message>
<xml_diff>
--- a/assets/data/Campo_Luna_Roja/Data_Riesgo_Prospectivo_MANUAL_Campo_Luna_Roja.xlsx
+++ b/assets/data/Campo_Luna_Roja/Data_Riesgo_Prospectivo_MANUAL_Campo_Luna_Roja.xlsx
@@ -522,7 +522,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -851,7 +851,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>

</xml_diff>